<commit_message>
02_ventas fechas ISO vs es-CL, 20_usuarios_dimensionado archivo de octubre, scripts cadena 10:30 y worklog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IRISCENE ENGINEERING CORPORATION SLU\Data Analytics Reporting Fractalia - CHILE\Miguel Paredes\Desarrollo\02. PYTHON\202_bot_jira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4158517F-DAFF-4217-B384-9415334B8A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F374861-BFCA-4070-9679-6411E5A03A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="489">
   <si>
     <t>Ticket</t>
   </si>
@@ -1164,13 +1164,346 @@
     <t>Migración ETL FCR de SSIS a python</t>
   </si>
   <si>
+    <t>Sí (30/09/2026 08:53)</t>
+  </si>
+  <si>
+    <t>518636</t>
+  </si>
+  <si>
+    <t>518727</t>
+  </si>
+  <si>
+    <t>518728</t>
+  </si>
+  <si>
+    <t>518729</t>
+  </si>
+  <si>
+    <t>Migración ETL EPA_WSP de SSIS a python</t>
+  </si>
+  <si>
+    <t>518637</t>
+  </si>
+  <si>
     <t>Desarrollo jefatura</t>
   </si>
   <si>
+    <t>518730</t>
+  </si>
+  <si>
     <t>Desarrollo lógica asunto_agrupado</t>
   </si>
   <si>
-    <t>Migración ETL EPA_WSP de SSIS a python</t>
+    <t>518731</t>
+  </si>
+  <si>
+    <t>518638</t>
+  </si>
+  <si>
+    <t>518732</t>
+  </si>
+  <si>
+    <t>518639</t>
+  </si>
+  <si>
+    <t>Sí (01/10/2026 09:05)</t>
+  </si>
+  <si>
+    <t>519124</t>
+  </si>
+  <si>
+    <t>519094</t>
+  </si>
+  <si>
+    <t>Curso Coursera</t>
+  </si>
+  <si>
+    <t>519125</t>
+  </si>
+  <si>
+    <t>Reunion: Migración bd_FFEE CXIOME KIT CONSULTING IA 15 (con Jair y Diego)</t>
+  </si>
+  <si>
+    <t>519095</t>
+  </si>
+  <si>
+    <t>Corrida ETL tráfico, calidad, usuarios chile (corrida manual por fuera de rango programado)</t>
+  </si>
+  <si>
+    <t>519126</t>
+  </si>
+  <si>
+    <t>Configuración servidor migración en dbeaver</t>
+  </si>
+  <si>
+    <t>519096</t>
+  </si>
+  <si>
+    <t>519097</t>
+  </si>
+  <si>
+    <t>Revision ETL de logueo</t>
+  </si>
+  <si>
+    <t>519127</t>
+  </si>
+  <si>
+    <t>519128</t>
+  </si>
+  <si>
+    <t>519098</t>
+  </si>
+  <si>
+    <t>519099</t>
+  </si>
+  <si>
+    <t>Reunion por solicitud nueva para el informe de correo, se necesita traer el número del caso mediante el cruce SF [ToAddress] - CorreoRegistro[ConversationID]</t>
+  </si>
+  <si>
+    <t>519129</t>
+  </si>
+  <si>
+    <t>519130</t>
+  </si>
+  <si>
+    <t>Sí (01/10/2026 17:16)</t>
+  </si>
+  <si>
+    <t>519236</t>
+  </si>
+  <si>
+    <t>Revision ETL de logueo: migración a pyhton, migración a microsoft graph, optimización de consultas en powerbi, programación de la tarea en el local</t>
+  </si>
+  <si>
+    <t>519300</t>
+  </si>
+  <si>
+    <t>519237</t>
+  </si>
+  <si>
+    <t>Revision de informes bi y origenes</t>
+  </si>
+  <si>
+    <t>519238</t>
+  </si>
+  <si>
+    <t>519301</t>
+  </si>
+  <si>
+    <t>519302</t>
+  </si>
+  <si>
+    <t>Sí (09/10/2026 07:46)</t>
+  </si>
+  <si>
+    <t>521869</t>
+  </si>
+  <si>
+    <t>Revisión archivos españa</t>
+  </si>
+  <si>
+    <t>521870</t>
+  </si>
+  <si>
+    <t>Revisión error acceso powerbi</t>
+  </si>
+  <si>
+    <t>522181</t>
+  </si>
+  <si>
+    <t>Migración de informes a microsoft graph</t>
+  </si>
+  <si>
+    <t>522182</t>
+  </si>
+  <si>
+    <t>Revision del proceso de ventas por caída, responsabilidad del asesor por cambio de nombre en unas de las columnas</t>
+  </si>
+  <si>
+    <t>521871</t>
+  </si>
+  <si>
+    <t>522183</t>
+  </si>
+  <si>
+    <t>522184</t>
+  </si>
+  <si>
+    <t>Reunion con Geoffery</t>
+  </si>
+  <si>
+    <t>521872</t>
+  </si>
+  <si>
+    <t>Migración de informes entre cuentas.</t>
+  </si>
+  <si>
+    <t>521873</t>
+  </si>
+  <si>
+    <t>Sí (09/10/2026 07:47)</t>
+  </si>
+  <si>
+    <t>521874</t>
+  </si>
+  <si>
+    <t>521875</t>
+  </si>
+  <si>
+    <t>521876</t>
+  </si>
+  <si>
+    <t>Desarrollo CDM</t>
+  </si>
+  <si>
+    <t>521877</t>
+  </si>
+  <si>
+    <t>Migración de informes bi</t>
+  </si>
+  <si>
+    <t>522185</t>
+  </si>
+  <si>
+    <t>521878</t>
+  </si>
+  <si>
+    <t>522186</t>
+  </si>
+  <si>
+    <t>Reunion con Jair</t>
+  </si>
+  <si>
+    <t>521879</t>
+  </si>
+  <si>
+    <t>522187</t>
+  </si>
+  <si>
+    <t>Reunion con Diana</t>
+  </si>
+  <si>
+    <t>522188</t>
+  </si>
+  <si>
+    <t>521880</t>
+  </si>
+  <si>
+    <t>Envío CDM</t>
+  </si>
+  <si>
+    <t>522189</t>
+  </si>
+  <si>
+    <t>522190</t>
+  </si>
+  <si>
+    <t>DSS-9811</t>
+  </si>
+  <si>
+    <t>Se reviso el informe y se detecta que se agregó una columna que no era parte del modelo y esto ocasionaba la caida.</t>
+  </si>
+  <si>
+    <t>521881</t>
+  </si>
+  <si>
+    <t>DSS-9814</t>
+  </si>
+  <si>
+    <t>Se reviso el informe y se detecta que en el archivo "análisis asignado" se agregó una columna que no era parte del modelo y esto ocasionaba la caida.</t>
+  </si>
+  <si>
+    <t>522191</t>
+  </si>
+  <si>
+    <t>DSS-9815</t>
+  </si>
+  <si>
+    <t>Factura setiembre</t>
+  </si>
+  <si>
+    <t>522192</t>
+  </si>
+  <si>
+    <t>Reunión Diego</t>
+  </si>
+  <si>
+    <t>522193</t>
+  </si>
+  <si>
+    <t>521882</t>
+  </si>
+  <si>
+    <t>DSS-9806</t>
+  </si>
+  <si>
+    <t>Atención ticket</t>
+  </si>
+  <si>
+    <t>522194</t>
+  </si>
+  <si>
+    <t>Factura setiembre, revision de indicadores de retenciones, no salia el mes de setiembre ni de agosto correctamente</t>
+  </si>
+  <si>
+    <t>521883</t>
+  </si>
+  <si>
+    <t>522195</t>
+  </si>
+  <si>
+    <t>Actualizacion termometro</t>
+  </si>
+  <si>
+    <t>522196</t>
+  </si>
+  <si>
+    <t>DSS-9780</t>
+  </si>
+  <si>
+    <t>Actualización multimétrico</t>
+  </si>
+  <si>
+    <t>522197</t>
+  </si>
+  <si>
+    <t>522198</t>
+  </si>
+  <si>
+    <t>522199</t>
+  </si>
+  <si>
+    <t>Sincronizacion de pc con onedrive</t>
+  </si>
+  <si>
+    <t>522200</t>
+  </si>
+  <si>
+    <t>521884</t>
+  </si>
+  <si>
+    <t>DSS-9785</t>
+  </si>
+  <si>
+    <t>Cambio en el campo de seguimiento [To Address], revision procedicimiento de seguimiento</t>
+  </si>
+  <si>
+    <t>522201</t>
+  </si>
+  <si>
+    <t>Impacto de cruce estapa silver</t>
+  </si>
+  <si>
+    <t>522202</t>
+  </si>
+  <si>
+    <t>522203</t>
+  </si>
+  <si>
+    <t>Actualización de cantidad de asesores por retenciones</t>
+  </si>
+  <si>
+    <t>Envio al cliente de factura setiembre</t>
   </si>
 </sst>
 </file>
@@ -1313,8 +1646,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H241" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:H241" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H303" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+  <autoFilter ref="A1:H303" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ticket"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="2"/>
@@ -1616,13 +1949,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H241"/>
+  <dimension ref="A1:H303"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="120.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="144.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
     <col min="7" max="7" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5703125" customWidth="1"/>
@@ -7191,8 +7524,14 @@
       <c r="E232" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="233" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="G232" t="s">
+        <v>375</v>
+      </c>
+      <c r="H232" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>8</v>
       </c>
@@ -7209,6 +7548,12 @@
       <c r="E233" s="5" t="s">
         <v>359</v>
       </c>
+      <c r="G233" t="s">
+        <v>375</v>
+      </c>
+      <c r="H233" t="s">
+        <v>377</v>
+      </c>
     </row>
     <row r="234" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
@@ -7227,24 +7572,36 @@
       <c r="E234" t="s">
         <v>340</v>
       </c>
+      <c r="G234" t="s">
+        <v>375</v>
+      </c>
+      <c r="H234" t="s">
+        <v>378</v>
+      </c>
     </row>
     <row r="235" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>8</v>
       </c>
       <c r="B235" s="1">
-        <v>46294.552083333336</v>
+        <v>46294.552083333343</v>
       </c>
       <c r="C235" s="3">
         <v>3.125E-2</v>
       </c>
       <c r="D235" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46294.583333333336</v>
+        <v>46294.583333333343</v>
       </c>
       <c r="E235" t="s">
         <v>374</v>
       </c>
+      <c r="G235" t="s">
+        <v>375</v>
+      </c>
+      <c r="H235" t="s">
+        <v>379</v>
+      </c>
     </row>
     <row r="236" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
@@ -7254,14 +7611,20 @@
         <v>46294.625</v>
       </c>
       <c r="C236" s="3">
-        <v>4.1666666666666664E-2</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="D236" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
         <v>46294.666666666664</v>
       </c>
       <c r="E236" t="s">
-        <v>377</v>
+        <v>380</v>
+      </c>
+      <c r="G236" t="s">
+        <v>375</v>
+      </c>
+      <c r="H236" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="237" spans="1:8" x14ac:dyDescent="0.25">
@@ -7269,17 +7632,23 @@
         <v>293</v>
       </c>
       <c r="B237" s="1">
-        <v>46294.666666666664</v>
+        <v>46294.666666666657</v>
       </c>
       <c r="C237" s="3">
-        <v>2.0833333333333332E-2</v>
+        <v>2.0833333333333329E-2</v>
       </c>
       <c r="D237" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46294.6875</v>
+        <v>46294.687499999993</v>
       </c>
       <c r="E237" t="s">
+        <v>382</v>
+      </c>
+      <c r="G237" t="s">
         <v>375</v>
+      </c>
+      <c r="H237" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="238" spans="1:8" x14ac:dyDescent="0.25">
@@ -7290,14 +7659,20 @@
         <v>46294.6875</v>
       </c>
       <c r="C238" s="3">
-        <v>2.0833333333333332E-2</v>
+        <v>2.0833333333333329E-2</v>
       </c>
       <c r="D238" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
         <v>46294.708333333336</v>
       </c>
       <c r="E238" t="s">
-        <v>376</v>
+        <v>384</v>
+      </c>
+      <c r="G238" t="s">
+        <v>375</v>
+      </c>
+      <c r="H238" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="239" spans="1:8" x14ac:dyDescent="0.25">
@@ -7305,53 +7680,1535 @@
         <v>12</v>
       </c>
       <c r="B239" s="1">
-        <v>46294.708333333336</v>
+        <v>46294.708333333343</v>
       </c>
       <c r="C239" s="3">
-        <v>1.3888888888888888E-2</v>
+        <v>1.388888888888889E-2</v>
       </c>
       <c r="D239" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46294.722222222226</v>
+        <v>46294.722222222234</v>
       </c>
       <c r="E239" t="s">
         <v>25</v>
       </c>
+      <c r="G239" t="s">
+        <v>375</v>
+      </c>
+      <c r="H239" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="240" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>8</v>
       </c>
       <c r="B240" s="1">
-        <v>46295.270833333336</v>
+        <v>46295.270833333343</v>
       </c>
       <c r="C240" s="3">
         <v>3.472222222222222E-3</v>
       </c>
       <c r="D240" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46295.274305555555</v>
+        <v>46295.274305555562</v>
       </c>
       <c r="E240" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G240" t="s">
+        <v>375</v>
+      </c>
+      <c r="H240" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>8</v>
       </c>
       <c r="B241" s="1">
-        <v>46295.274305555555</v>
+        <v>46295.274305555547</v>
       </c>
       <c r="C241" s="3">
-        <v>0.10069444444444445</v>
+        <v>0.10069444444444441</v>
       </c>
       <c r="D241" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46295.375</v>
+        <v>46295.374999999993</v>
       </c>
       <c r="E241" t="s">
-        <v>377</v>
+        <v>380</v>
+      </c>
+      <c r="G241" t="s">
+        <v>375</v>
+      </c>
+      <c r="H241" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>12</v>
+      </c>
+      <c r="B242" s="1">
+        <v>46295.354166666657</v>
+      </c>
+      <c r="C242" s="3">
+        <v>2.2916666666666669E-2</v>
+      </c>
+      <c r="D242" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.377083333326</v>
+      </c>
+      <c r="E242" t="s">
+        <v>15</v>
+      </c>
+      <c r="G242" t="s">
+        <v>389</v>
+      </c>
+      <c r="H242" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>8</v>
+      </c>
+      <c r="B243" s="1">
+        <v>46295.377083333333</v>
+      </c>
+      <c r="C243" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D243" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.384027777778</v>
+      </c>
+      <c r="E243" t="s">
+        <v>329</v>
+      </c>
+      <c r="G243" t="s">
+        <v>389</v>
+      </c>
+      <c r="H243" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>8</v>
+      </c>
+      <c r="B244" s="1">
+        <v>46295.384027777778</v>
+      </c>
+      <c r="C244" s="3">
+        <v>3.2638888888888891E-2</v>
+      </c>
+      <c r="D244" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.416666666664</v>
+      </c>
+      <c r="E244" t="s">
+        <v>392</v>
+      </c>
+      <c r="G244" t="s">
+        <v>389</v>
+      </c>
+      <c r="H244" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>12</v>
+      </c>
+      <c r="B245" s="1">
+        <v>46295.4375</v>
+      </c>
+      <c r="C245" s="3">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D245" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.520833333336</v>
+      </c>
+      <c r="E245" t="s">
+        <v>394</v>
+      </c>
+      <c r="G245" t="s">
+        <v>389</v>
+      </c>
+      <c r="H245" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>8</v>
+      </c>
+      <c r="B246" s="1">
+        <v>46295.520833333343</v>
+      </c>
+      <c r="C246" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D246" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.562500000007</v>
+      </c>
+      <c r="E246" t="s">
+        <v>396</v>
+      </c>
+      <c r="G246" t="s">
+        <v>389</v>
+      </c>
+      <c r="H246" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>12</v>
+      </c>
+      <c r="B247" s="1">
+        <v>46295.5625</v>
+      </c>
+      <c r="C247" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D247" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.583333333336</v>
+      </c>
+      <c r="E247" t="s">
+        <v>398</v>
+      </c>
+      <c r="G247" t="s">
+        <v>389</v>
+      </c>
+      <c r="H247" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>8</v>
+      </c>
+      <c r="B248" s="1">
+        <v>46295.625</v>
+      </c>
+      <c r="C248" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D248" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.631944444445</v>
+      </c>
+      <c r="E248" t="s">
+        <v>329</v>
+      </c>
+      <c r="G248" t="s">
+        <v>389</v>
+      </c>
+      <c r="H248" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>8</v>
+      </c>
+      <c r="B249" s="1">
+        <v>46295.631944444453</v>
+      </c>
+      <c r="C249" s="3">
+        <v>3.4722222222222217E-2</v>
+      </c>
+      <c r="D249" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.666666666672</v>
+      </c>
+      <c r="E249" t="s">
+        <v>401</v>
+      </c>
+      <c r="G249" t="s">
+        <v>389</v>
+      </c>
+      <c r="H249" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>12</v>
+      </c>
+      <c r="B250" s="1">
+        <v>46295.666666666657</v>
+      </c>
+      <c r="C250" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D250" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46295.708333333321</v>
+      </c>
+      <c r="E250" t="s">
+        <v>25</v>
+      </c>
+      <c r="G250" t="s">
+        <v>389</v>
+      </c>
+      <c r="H250" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>8</v>
+      </c>
+      <c r="B251" s="1">
+        <v>46296.270833333343</v>
+      </c>
+      <c r="C251" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D251" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.274305555562</v>
+      </c>
+      <c r="E251" t="s">
+        <v>9</v>
+      </c>
+      <c r="G251" t="s">
+        <v>389</v>
+      </c>
+      <c r="H251" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>8</v>
+      </c>
+      <c r="B252" s="1">
+        <v>46296.274305555547</v>
+      </c>
+      <c r="C252" s="3">
+        <v>7.2916666666666671E-2</v>
+      </c>
+      <c r="D252" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.347222222212</v>
+      </c>
+      <c r="E252" t="s">
+        <v>401</v>
+      </c>
+      <c r="G252" t="s">
+        <v>389</v>
+      </c>
+      <c r="H252" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>8</v>
+      </c>
+      <c r="B253" s="1">
+        <v>46296.347222222219</v>
+      </c>
+      <c r="C253" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D253" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.354166666664</v>
+      </c>
+      <c r="E253" t="s">
+        <v>406</v>
+      </c>
+      <c r="G253" t="s">
+        <v>389</v>
+      </c>
+      <c r="H253" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>8</v>
+      </c>
+      <c r="B254" s="1">
+        <v>46296.354166666657</v>
+      </c>
+      <c r="C254" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D254" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.374999999993</v>
+      </c>
+      <c r="E254" t="s">
+        <v>401</v>
+      </c>
+      <c r="G254" t="s">
+        <v>389</v>
+      </c>
+      <c r="H254" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>12</v>
+      </c>
+      <c r="B255" s="1">
+        <v>46296.375</v>
+      </c>
+      <c r="C255" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D255" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.395833333336</v>
+      </c>
+      <c r="E255" t="s">
+        <v>15</v>
+      </c>
+      <c r="G255" t="s">
+        <v>409</v>
+      </c>
+      <c r="H255" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>8</v>
+      </c>
+      <c r="B256" s="1">
+        <v>46296.395833333343</v>
+      </c>
+      <c r="C256" s="3">
+        <v>0.14583333333333329</v>
+      </c>
+      <c r="D256" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.541666666679</v>
+      </c>
+      <c r="E256" t="s">
+        <v>411</v>
+      </c>
+      <c r="G256" t="s">
+        <v>409</v>
+      </c>
+      <c r="H256" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>8</v>
+      </c>
+      <c r="B257" s="1">
+        <v>46296.541666666657</v>
+      </c>
+      <c r="C257" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D257" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.555555555547</v>
+      </c>
+      <c r="E257" t="s">
+        <v>155</v>
+      </c>
+      <c r="G257" t="s">
+        <v>409</v>
+      </c>
+      <c r="H257" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
+        <v>12</v>
+      </c>
+      <c r="B258" s="1">
+        <v>46296.555555555547</v>
+      </c>
+      <c r="C258" s="3">
+        <v>2.777777777777778E-2</v>
+      </c>
+      <c r="D258" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.583333333328</v>
+      </c>
+      <c r="E258" t="s">
+        <v>414</v>
+      </c>
+      <c r="G258" t="s">
+        <v>409</v>
+      </c>
+      <c r="H258" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>12</v>
+      </c>
+      <c r="B259" s="1">
+        <v>46296.625</v>
+      </c>
+      <c r="C259" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D259" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.666666666664</v>
+      </c>
+      <c r="E259" t="s">
+        <v>414</v>
+      </c>
+      <c r="G259" t="s">
+        <v>409</v>
+      </c>
+      <c r="H259" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>12</v>
+      </c>
+      <c r="B260" s="1">
+        <v>46296.666666666657</v>
+      </c>
+      <c r="C260" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="D260" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46296.71666666666</v>
+      </c>
+      <c r="E260" t="s">
+        <v>25</v>
+      </c>
+      <c r="G260" t="s">
+        <v>409</v>
+      </c>
+      <c r="H260" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>8</v>
+      </c>
+      <c r="B261" s="1">
+        <v>46300.270833333343</v>
+      </c>
+      <c r="C261" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D261" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.274305555562</v>
+      </c>
+      <c r="E261" t="s">
+        <v>9</v>
+      </c>
+      <c r="G261" t="s">
+        <v>418</v>
+      </c>
+      <c r="H261" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>12</v>
+      </c>
+      <c r="B262" s="1">
+        <v>46300.274305555547</v>
+      </c>
+      <c r="C262" s="3">
+        <v>1.7361111111111108E-2</v>
+      </c>
+      <c r="D262" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.291666666657</v>
+      </c>
+      <c r="E262" t="s">
+        <v>420</v>
+      </c>
+      <c r="G262" t="s">
+        <v>418</v>
+      </c>
+      <c r="H262" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
+        <v>12</v>
+      </c>
+      <c r="B263" s="1">
+        <v>46300.291666666657</v>
+      </c>
+      <c r="C263" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D263" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.312499999993</v>
+      </c>
+      <c r="E263" t="s">
+        <v>422</v>
+      </c>
+      <c r="G263" t="s">
+        <v>418</v>
+      </c>
+      <c r="H263" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>12</v>
+      </c>
+      <c r="B264" s="1">
+        <v>46300.3125</v>
+      </c>
+      <c r="C264" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D264" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.354166666664</v>
+      </c>
+      <c r="E264" t="s">
+        <v>424</v>
+      </c>
+      <c r="G264" t="s">
+        <v>418</v>
+      </c>
+      <c r="H264" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
+        <v>8</v>
+      </c>
+      <c r="B265" s="1">
+        <v>46300.354166666657</v>
+      </c>
+      <c r="C265" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D265" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.374999999993</v>
+      </c>
+      <c r="E265" t="s">
+        <v>426</v>
+      </c>
+      <c r="G265" t="s">
+        <v>418</v>
+      </c>
+      <c r="H265" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>12</v>
+      </c>
+      <c r="B266" s="1">
+        <v>46300.375</v>
+      </c>
+      <c r="C266" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D266" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.385416666664</v>
+      </c>
+      <c r="E266" t="s">
+        <v>15</v>
+      </c>
+      <c r="G266" t="s">
+        <v>418</v>
+      </c>
+      <c r="H266" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>12</v>
+      </c>
+      <c r="B267" s="1">
+        <v>46300.385416666657</v>
+      </c>
+      <c r="C267" s="3">
+        <v>3.125E-2</v>
+      </c>
+      <c r="D267" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.416666666657</v>
+      </c>
+      <c r="E267" t="s">
+        <v>424</v>
+      </c>
+      <c r="G267" t="s">
+        <v>418</v>
+      </c>
+      <c r="H267" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>8</v>
+      </c>
+      <c r="B268" s="1">
+        <v>46300.416666666657</v>
+      </c>
+      <c r="C268" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D268" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.458333333321</v>
+      </c>
+      <c r="E268" t="s">
+        <v>430</v>
+      </c>
+      <c r="G268" t="s">
+        <v>418</v>
+      </c>
+      <c r="H268" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>12</v>
+      </c>
+      <c r="B269" s="1">
+        <v>46300.458333333343</v>
+      </c>
+      <c r="C269" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="D269" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.583333333343</v>
+      </c>
+      <c r="E269" t="s">
+        <v>432</v>
+      </c>
+      <c r="G269" t="s">
+        <v>418</v>
+      </c>
+      <c r="H269" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>12</v>
+      </c>
+      <c r="B270" s="1">
+        <v>46300.625</v>
+      </c>
+      <c r="C270" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D270" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.666666666664</v>
+      </c>
+      <c r="E270" t="s">
+        <v>424</v>
+      </c>
+      <c r="G270" t="s">
+        <v>434</v>
+      </c>
+      <c r="H270" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>12</v>
+      </c>
+      <c r="B271" s="1">
+        <v>46300.666666666657</v>
+      </c>
+      <c r="C271" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="D271" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46300.71666666666</v>
+      </c>
+      <c r="E271" t="s">
+        <v>25</v>
+      </c>
+      <c r="G271" t="s">
+        <v>434</v>
+      </c>
+      <c r="H271" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>8</v>
+      </c>
+      <c r="B272" s="1">
+        <v>46301.270833333343</v>
+      </c>
+      <c r="C272" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D272" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.274305555562</v>
+      </c>
+      <c r="E272" t="s">
+        <v>9</v>
+      </c>
+      <c r="G272" t="s">
+        <v>434</v>
+      </c>
+      <c r="H272" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>8</v>
+      </c>
+      <c r="B273" s="1">
+        <v>46301.274305555547</v>
+      </c>
+      <c r="C273" s="3">
+        <v>1.7361111111111108E-2</v>
+      </c>
+      <c r="D273" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.291666666657</v>
+      </c>
+      <c r="E273" t="s">
+        <v>438</v>
+      </c>
+      <c r="G273" t="s">
+        <v>434</v>
+      </c>
+      <c r="H273" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>12</v>
+      </c>
+      <c r="B274" s="1">
+        <v>46301.291666666657</v>
+      </c>
+      <c r="C274" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D274" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.312499999993</v>
+      </c>
+      <c r="E274" t="s">
+        <v>440</v>
+      </c>
+      <c r="G274" t="s">
+        <v>434</v>
+      </c>
+      <c r="H274" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>8</v>
+      </c>
+      <c r="B275" s="1">
+        <v>46301.3125</v>
+      </c>
+      <c r="C275" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D275" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.354166666664</v>
+      </c>
+      <c r="E275" t="s">
+        <v>438</v>
+      </c>
+      <c r="G275" t="s">
+        <v>434</v>
+      </c>
+      <c r="H275" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>12</v>
+      </c>
+      <c r="B276" s="1">
+        <v>46301.354166666657</v>
+      </c>
+      <c r="C276" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D276" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.374999999993</v>
+      </c>
+      <c r="E276" t="s">
+        <v>15</v>
+      </c>
+      <c r="G276" t="s">
+        <v>434</v>
+      </c>
+      <c r="H276" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>8</v>
+      </c>
+      <c r="B277" s="1">
+        <v>46301.375</v>
+      </c>
+      <c r="C277" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D277" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.395833333336</v>
+      </c>
+      <c r="E277" t="s">
+        <v>444</v>
+      </c>
+      <c r="G277" t="s">
+        <v>434</v>
+      </c>
+      <c r="H277" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>8</v>
+      </c>
+      <c r="B278" s="1">
+        <v>46301.395833333343</v>
+      </c>
+      <c r="C278" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D278" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.458333333343</v>
+      </c>
+      <c r="E278" t="s">
+        <v>438</v>
+      </c>
+      <c r="G278" t="s">
+        <v>434</v>
+      </c>
+      <c r="H278" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>8</v>
+      </c>
+      <c r="B279" s="1">
+        <v>46301.458333333343</v>
+      </c>
+      <c r="C279" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D279" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.479166666679</v>
+      </c>
+      <c r="E279" t="s">
+        <v>447</v>
+      </c>
+      <c r="G279" t="s">
+        <v>434</v>
+      </c>
+      <c r="H279" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>8</v>
+      </c>
+      <c r="B280" s="1">
+        <v>46301.479166666657</v>
+      </c>
+      <c r="C280" s="3">
+        <v>0.1041666666666667</v>
+      </c>
+      <c r="D280" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.583333333321</v>
+      </c>
+      <c r="E280" t="s">
+        <v>438</v>
+      </c>
+      <c r="G280" t="s">
+        <v>434</v>
+      </c>
+      <c r="H280" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>8</v>
+      </c>
+      <c r="B281" s="1">
+        <v>46301.625</v>
+      </c>
+      <c r="C281" s="3">
+        <v>0.10069444444444441</v>
+      </c>
+      <c r="D281" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46301.725694444445</v>
+      </c>
+      <c r="E281" t="s">
+        <v>450</v>
+      </c>
+      <c r="G281" t="s">
+        <v>434</v>
+      </c>
+      <c r="H281" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>8</v>
+      </c>
+      <c r="B282" s="1">
+        <v>46302.270833333343</v>
+      </c>
+      <c r="C282" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D282" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.274305555562</v>
+      </c>
+      <c r="E282" t="s">
+        <v>9</v>
+      </c>
+      <c r="G282" t="s">
+        <v>434</v>
+      </c>
+      <c r="H282" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>453</v>
+      </c>
+      <c r="B283" s="1">
+        <v>46302.274305555547</v>
+      </c>
+      <c r="C283" s="3">
+        <v>1.7361111111111108E-2</v>
+      </c>
+      <c r="D283" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.291666666657</v>
+      </c>
+      <c r="E283" t="s">
+        <v>454</v>
+      </c>
+      <c r="G283" t="s">
+        <v>434</v>
+      </c>
+      <c r="H283" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>456</v>
+      </c>
+      <c r="B284" s="1">
+        <v>46302.291666666657</v>
+      </c>
+      <c r="C284" s="3">
+        <v>2.4305555555555559E-2</v>
+      </c>
+      <c r="D284" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.315972222212</v>
+      </c>
+      <c r="E284" t="s">
+        <v>457</v>
+      </c>
+      <c r="G284" t="s">
+        <v>434</v>
+      </c>
+      <c r="H284" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>459</v>
+      </c>
+      <c r="B285" s="1">
+        <v>46302.315972222219</v>
+      </c>
+      <c r="C285" s="3">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="D285" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.354166666664</v>
+      </c>
+      <c r="E285" t="s">
+        <v>460</v>
+      </c>
+      <c r="G285" t="s">
+        <v>434</v>
+      </c>
+      <c r="H285" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>12</v>
+      </c>
+      <c r="B286" s="1">
+        <v>46302.354166666657</v>
+      </c>
+      <c r="C286" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D286" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.374999999993</v>
+      </c>
+      <c r="E286" t="s">
+        <v>462</v>
+      </c>
+      <c r="G286" t="s">
+        <v>434</v>
+      </c>
+      <c r="H286" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>12</v>
+      </c>
+      <c r="B287" s="1">
+        <v>46302.375</v>
+      </c>
+      <c r="C287" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D287" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.395833333336</v>
+      </c>
+      <c r="E287" t="s">
+        <v>15</v>
+      </c>
+      <c r="G287" t="s">
+        <v>434</v>
+      </c>
+      <c r="H287" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>465</v>
+      </c>
+      <c r="B288" s="1">
+        <v>46302.395833333343</v>
+      </c>
+      <c r="C288" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D288" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.399305555562</v>
+      </c>
+      <c r="E288" t="s">
+        <v>466</v>
+      </c>
+      <c r="G288" t="s">
+        <v>434</v>
+      </c>
+      <c r="H288" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>459</v>
+      </c>
+      <c r="B289" s="1">
+        <v>46302.399305555547</v>
+      </c>
+      <c r="C289" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="D289" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.524305555547</v>
+      </c>
+      <c r="E289" t="s">
+        <v>468</v>
+      </c>
+      <c r="G289" t="s">
+        <v>434</v>
+      </c>
+      <c r="H289" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>8</v>
+      </c>
+      <c r="B290" s="1">
+        <v>46302.524305555547</v>
+      </c>
+      <c r="C290" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D290" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.531249999993</v>
+      </c>
+      <c r="E290" t="s">
+        <v>329</v>
+      </c>
+      <c r="G290" t="s">
+        <v>434</v>
+      </c>
+      <c r="H290" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>8</v>
+      </c>
+      <c r="B291" s="1">
+        <v>46302.53125</v>
+      </c>
+      <c r="C291" s="3">
+        <v>3.125E-2</v>
+      </c>
+      <c r="D291" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.5625</v>
+      </c>
+      <c r="E291" t="s">
+        <v>471</v>
+      </c>
+      <c r="G291" t="s">
+        <v>434</v>
+      </c>
+      <c r="H291" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>473</v>
+      </c>
+      <c r="B292" s="1">
+        <v>46302.5625</v>
+      </c>
+      <c r="C292" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D292" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.583333333336</v>
+      </c>
+      <c r="E292" t="s">
+        <v>474</v>
+      </c>
+      <c r="G292" t="s">
+        <v>434</v>
+      </c>
+      <c r="H292" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>473</v>
+      </c>
+      <c r="B293" s="1">
+        <v>46302.625</v>
+      </c>
+      <c r="C293" s="3">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D293" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46302.708333333336</v>
+      </c>
+      <c r="E293" t="s">
+        <v>474</v>
+      </c>
+      <c r="G293" t="s">
+        <v>434</v>
+      </c>
+      <c r="H293" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
+        <v>8</v>
+      </c>
+      <c r="B294" s="1">
+        <v>46303.270833333343</v>
+      </c>
+      <c r="C294" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D294" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46303.274305555562</v>
+      </c>
+      <c r="E294" t="s">
+        <v>9</v>
+      </c>
+      <c r="G294" t="s">
+        <v>434</v>
+      </c>
+      <c r="H294" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>8</v>
+      </c>
+      <c r="B295" s="1">
+        <v>46303.270833333343</v>
+      </c>
+      <c r="C295" s="3">
+        <v>0.14583333333333329</v>
+      </c>
+      <c r="D295" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46303.416666666679</v>
+      </c>
+      <c r="E295" t="s">
+        <v>478</v>
+      </c>
+      <c r="G295" t="s">
+        <v>434</v>
+      </c>
+      <c r="H295" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>473</v>
+      </c>
+      <c r="B296" s="1">
+        <v>46303.416666666657</v>
+      </c>
+      <c r="C296" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D296" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46303.479166666657</v>
+      </c>
+      <c r="E296" t="s">
+        <v>474</v>
+      </c>
+      <c r="G296" t="s">
+        <v>434</v>
+      </c>
+      <c r="H296" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>481</v>
+      </c>
+      <c r="B297" s="1">
+        <v>46303.479166666657</v>
+      </c>
+      <c r="C297" s="3">
+        <v>0.1041666666666667</v>
+      </c>
+      <c r="D297" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46303.583333333321</v>
+      </c>
+      <c r="E297" t="s">
+        <v>482</v>
+      </c>
+      <c r="G297" t="s">
+        <v>434</v>
+      </c>
+      <c r="H297" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>481</v>
+      </c>
+      <c r="B298" s="1">
+        <v>46303.625</v>
+      </c>
+      <c r="C298" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D298" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46303.666666666664</v>
+      </c>
+      <c r="E298" t="s">
+        <v>484</v>
+      </c>
+      <c r="G298" t="s">
+        <v>434</v>
+      </c>
+      <c r="H298" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>12</v>
+      </c>
+      <c r="B299" s="1">
+        <v>46303.666666666657</v>
+      </c>
+      <c r="C299" s="3">
+        <v>5.6944444444444443E-2</v>
+      </c>
+      <c r="D299" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46303.723611111098</v>
+      </c>
+      <c r="E299" t="s">
+        <v>25</v>
+      </c>
+      <c r="G299" t="s">
+        <v>434</v>
+      </c>
+      <c r="H299" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>8</v>
+      </c>
+      <c r="B300" s="1">
+        <v>46304.270833333336</v>
+      </c>
+      <c r="C300" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D300" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.274305555555</v>
+      </c>
+      <c r="E300" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>459</v>
+      </c>
+      <c r="B301" s="1">
+        <v>46304.274305555555</v>
+      </c>
+      <c r="C301" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D301" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.277777777774</v>
+      </c>
+      <c r="E301" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
+        <v>459</v>
+      </c>
+      <c r="B302" s="1">
+        <v>46304.326388888891</v>
+      </c>
+      <c r="C302" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D302" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.329861111109</v>
+      </c>
+      <c r="E302" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
+        <v>481</v>
+      </c>
+      <c r="B303" s="1">
+        <v>46304.329861111109</v>
+      </c>
+      <c r="C303" s="3">
+        <v>0</v>
+      </c>
+      <c r="D303" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.329861111109</v>
+      </c>
+      <c r="E303" t="s">
+        <v>484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualziación de correos y epa
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IRISCENE ENGINEERING CORPORATION SLU\Data Analytics Reporting Fractalia - CHILE\Miguel Paredes\Desarrollo\02. PYTHON\202_bot_jira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F374861-BFCA-4070-9679-6411E5A03A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8563D9EC-C391-460D-8245-61AAEDFC46DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="534">
   <si>
     <t>Ticket</t>
   </si>
@@ -1500,10 +1500,147 @@
     <t>522203</t>
   </si>
   <si>
+    <t>Sí (13/10/2026 08:21)</t>
+  </si>
+  <si>
+    <t>522941</t>
+  </si>
+  <si>
     <t>Actualización de cantidad de asesores por retenciones</t>
   </si>
   <si>
+    <t>522888</t>
+  </si>
+  <si>
+    <t>Desarrollo multimétrico</t>
+  </si>
+  <si>
+    <t>522889</t>
+  </si>
+  <si>
     <t>Envio al cliente de factura setiembre</t>
+  </si>
+  <si>
+    <t>522942</t>
+  </si>
+  <si>
+    <t>522890</t>
+  </si>
+  <si>
+    <t>522943</t>
+  </si>
+  <si>
+    <t>Reunion Jair</t>
+  </si>
+  <si>
+    <t>522891</t>
+  </si>
+  <si>
+    <t>Reunion Oscar</t>
+  </si>
+  <si>
+    <t>522892</t>
+  </si>
+  <si>
+    <t>Revisión de procesos por truncamiento trafico y portal comercial, se detecta que ambos tienen problemas en las contraseñas se necesitaba renovar</t>
+  </si>
+  <si>
+    <t>522893</t>
+  </si>
+  <si>
+    <t>522944</t>
+  </si>
+  <si>
+    <t>522945</t>
+  </si>
+  <si>
+    <t>Migración OneDrive</t>
+  </si>
+  <si>
+    <t>522894</t>
+  </si>
+  <si>
+    <t>522946</t>
+  </si>
+  <si>
+    <t>Llamada con Oscar para brindarle la ruta de los archivos en el sharepoint</t>
+  </si>
+  <si>
+    <t>522947</t>
+  </si>
+  <si>
+    <t>Reunión de parametros para el multimétrico</t>
+  </si>
+  <si>
+    <t>522895</t>
+  </si>
+  <si>
+    <t>522948</t>
+  </si>
+  <si>
+    <t>Levantamiento de informes caídos powerbi</t>
+  </si>
+  <si>
+    <t>522896</t>
+  </si>
+  <si>
+    <t>522949</t>
+  </si>
+  <si>
+    <t>522950</t>
+  </si>
+  <si>
+    <t>Revisión informes retenciones, dado que no sale el mes de octubre</t>
+  </si>
+  <si>
+    <t>522897</t>
+  </si>
+  <si>
+    <t>Optimización de query informe OpenAi</t>
+  </si>
+  <si>
+    <t>Optimización de query informe OpenAi y asistencia
+Migración de cuenta de analistas a reporting
+Optimización de query's</t>
+  </si>
+  <si>
+    <t>Reunión Diana definir parametros de trabajo</t>
+  </si>
+  <si>
+    <t>DSS-9833</t>
+  </si>
+  <si>
+    <t>Se adjunto el archivosolicitado por katherine vasquez</t>
+  </si>
+  <si>
+    <t>Revision de procesos bi, no carga los registros actuales</t>
+  </si>
+  <si>
+    <t>Revisión de informe asistencia 2023</t>
+  </si>
+  <si>
+    <t>Envio de cambios SM</t>
+  </si>
+  <si>
+    <t>DSS-9839</t>
+  </si>
+  <si>
+    <t>Se modifico la vista en el informe, se modifico el campo fecha.</t>
+  </si>
+  <si>
+    <t>DSS-9834</t>
+  </si>
+  <si>
+    <t>Se realizo las consultas respectivas y coordinaciones sin llegar a encontrar los registros del año 2023</t>
+  </si>
+  <si>
+    <t>Envio de cambios SM, revisión de malos datos por parte de triadas, gestión de coordinación y modificación del archivo</t>
+  </si>
+  <si>
+    <t>Acualización de archivo de place</t>
+  </si>
+  <si>
+    <t>Corregir la jefatura en el informe de correo</t>
   </si>
 </sst>
 </file>
@@ -1566,7 +1703,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1578,6 +1715,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1595,16 +1744,16 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <top style="thin">
+        <bottom style="thin">
           <color auto="1"/>
-        </top>
+        </bottom>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
+        <top style="thin">
           <color auto="1"/>
-        </bottom>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -1646,8 +1795,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H303" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:H303" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H334" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="3" tableBorderDxfId="4">
+  <autoFilter ref="A1:H334" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ticket"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="2"/>
@@ -1949,7 +2098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H303"/>
+  <dimension ref="A1:H334"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
@@ -9144,17 +9293,23 @@
         <v>8</v>
       </c>
       <c r="B300" s="1">
-        <v>46304.270833333336</v>
+        <v>46304.270833333343</v>
       </c>
       <c r="C300" s="3">
         <v>3.472222222222222E-3</v>
       </c>
       <c r="D300" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46304.274305555555</v>
+        <v>46304.274305555562</v>
       </c>
       <c r="E300" t="s">
         <v>9</v>
+      </c>
+      <c r="G300" t="s">
+        <v>487</v>
+      </c>
+      <c r="H300" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="301" spans="1:8" x14ac:dyDescent="0.25">
@@ -9162,53 +9317,725 @@
         <v>459</v>
       </c>
       <c r="B301" s="1">
-        <v>46304.274305555555</v>
+        <v>46304.274305555547</v>
       </c>
       <c r="C301" s="3">
         <v>3.472222222222222E-3</v>
       </c>
       <c r="D301" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46304.277777777774</v>
+        <v>46304.277777777766</v>
       </c>
       <c r="E301" t="s">
+        <v>489</v>
+      </c>
+      <c r="G301" t="s">
         <v>487</v>
+      </c>
+      <c r="H301" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="302" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>459</v>
+        <v>473</v>
       </c>
       <c r="B302" s="1">
+        <v>46304.277777777781</v>
+      </c>
+      <c r="C302" s="3">
+        <v>4.8611111111111112E-2</v>
+      </c>
+      <c r="D302" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
         <v>46304.326388888891</v>
       </c>
-      <c r="C302" s="3">
-        <v>3.472222222222222E-3</v>
-      </c>
-      <c r="D302" s="3">
-        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46304.329861111109</v>
-      </c>
       <c r="E302" t="s">
-        <v>488</v>
+        <v>491</v>
+      </c>
+      <c r="G302" t="s">
+        <v>487</v>
+      </c>
+      <c r="H302" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="303" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
+        <v>459</v>
+      </c>
+      <c r="B303" s="1">
+        <v>46304.326388888891</v>
+      </c>
+      <c r="C303" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D303" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.329861111109</v>
+      </c>
+      <c r="E303" t="s">
+        <v>493</v>
+      </c>
+      <c r="G303" t="s">
+        <v>487</v>
+      </c>
+      <c r="H303" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
         <v>481</v>
       </c>
-      <c r="B303" s="1">
+      <c r="B304" s="1">
         <v>46304.329861111109</v>
       </c>
-      <c r="C303" s="3">
-        <v>0</v>
-      </c>
-      <c r="D303" s="3">
-        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46304.329861111109</v>
-      </c>
-      <c r="E303" t="s">
+      <c r="C304" s="3">
+        <v>4.5138888888888888E-2</v>
+      </c>
+      <c r="D304" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.375</v>
+      </c>
+      <c r="E304" t="s">
         <v>484</v>
+      </c>
+      <c r="G304" t="s">
+        <v>487</v>
+      </c>
+      <c r="H304" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>12</v>
+      </c>
+      <c r="B305" s="1">
+        <v>46304.375</v>
+      </c>
+      <c r="C305" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D305" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.388888888891</v>
+      </c>
+      <c r="E305" t="s">
+        <v>15</v>
+      </c>
+      <c r="G305" t="s">
+        <v>487</v>
+      </c>
+      <c r="H305" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>12</v>
+      </c>
+      <c r="B306" s="1">
+        <v>46304.388888888891</v>
+      </c>
+      <c r="C306" s="3">
+        <v>2.777777777777778E-2</v>
+      </c>
+      <c r="D306" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.416666666672</v>
+      </c>
+      <c r="E306" t="s">
+        <v>497</v>
+      </c>
+      <c r="G306" t="s">
+        <v>487</v>
+      </c>
+      <c r="H306" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>12</v>
+      </c>
+      <c r="B307" s="1">
+        <v>46304.416666666657</v>
+      </c>
+      <c r="C307" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D307" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.458333333321</v>
+      </c>
+      <c r="E307" t="s">
+        <v>499</v>
+      </c>
+      <c r="G307" t="s">
+        <v>487</v>
+      </c>
+      <c r="H307" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>8</v>
+      </c>
+      <c r="B308" s="1">
+        <v>46304.458333333343</v>
+      </c>
+      <c r="C308" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D308" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.500000000007</v>
+      </c>
+      <c r="E308" t="s">
+        <v>501</v>
+      </c>
+      <c r="G308" t="s">
+        <v>487</v>
+      </c>
+      <c r="H308" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
+        <v>8</v>
+      </c>
+      <c r="B309" s="1">
+        <v>46304.5</v>
+      </c>
+      <c r="C309" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D309" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.506944444445</v>
+      </c>
+      <c r="E309" t="s">
+        <v>329</v>
+      </c>
+      <c r="G309" t="s">
+        <v>487</v>
+      </c>
+      <c r="H309" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A310" t="s">
+        <v>8</v>
+      </c>
+      <c r="B310" s="1">
+        <v>46274.506944444453</v>
+      </c>
+      <c r="C310" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D310" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.527777777788</v>
+      </c>
+      <c r="E310" t="s">
+        <v>155</v>
+      </c>
+      <c r="G310" t="s">
+        <v>487</v>
+      </c>
+      <c r="H310" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A311" t="s">
+        <v>12</v>
+      </c>
+      <c r="B311" s="1">
+        <v>46304.527777777781</v>
+      </c>
+      <c r="C311" s="3">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D311" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.583333333336</v>
+      </c>
+      <c r="E311" t="s">
+        <v>505</v>
+      </c>
+      <c r="G311" t="s">
+        <v>487</v>
+      </c>
+      <c r="H311" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A312" t="s">
+        <v>12</v>
+      </c>
+      <c r="B312" s="1">
+        <v>46304.625</v>
+      </c>
+      <c r="C312" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D312" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.666666666664</v>
+      </c>
+      <c r="E312" t="s">
+        <v>505</v>
+      </c>
+      <c r="G312" t="s">
+        <v>487</v>
+      </c>
+      <c r="H312" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A313" t="s">
+        <v>12</v>
+      </c>
+      <c r="B313" s="1">
+        <v>46304.666666666657</v>
+      </c>
+      <c r="C313" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D313" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.687499999993</v>
+      </c>
+      <c r="E313" t="s">
+        <v>508</v>
+      </c>
+      <c r="G313" t="s">
+        <v>487</v>
+      </c>
+      <c r="H313" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
+        <v>473</v>
+      </c>
+      <c r="B314" s="1">
+        <v>46304.6875</v>
+      </c>
+      <c r="C314" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D314" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46304.708333333336</v>
+      </c>
+      <c r="E314" t="s">
+        <v>510</v>
+      </c>
+      <c r="G314" t="s">
+        <v>487</v>
+      </c>
+      <c r="H314" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A315" t="s">
+        <v>8</v>
+      </c>
+      <c r="B315" s="1">
+        <v>46308.270833333343</v>
+      </c>
+      <c r="C315" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D315" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.274305555562</v>
+      </c>
+      <c r="E315" t="s">
+        <v>9</v>
+      </c>
+      <c r="G315" t="s">
+        <v>487</v>
+      </c>
+      <c r="H315" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A316" t="s">
+        <v>8</v>
+      </c>
+      <c r="B316" s="1">
+        <v>46308.270833333343</v>
+      </c>
+      <c r="C316" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D316" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.291666666679</v>
+      </c>
+      <c r="E316" t="s">
+        <v>513</v>
+      </c>
+      <c r="G316" t="s">
+        <v>487</v>
+      </c>
+      <c r="H316" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A317" t="s">
+        <v>12</v>
+      </c>
+      <c r="B317" s="1">
+        <v>46308.291666666657</v>
+      </c>
+      <c r="C317" s="3">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="D317" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.329861111102</v>
+      </c>
+      <c r="E317" t="s">
+        <v>505</v>
+      </c>
+      <c r="G317" t="s">
+        <v>487</v>
+      </c>
+      <c r="H317" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="318" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A318" t="s">
+        <v>8</v>
+      </c>
+      <c r="B318" s="1">
+        <v>46308.329861111109</v>
+      </c>
+      <c r="C318" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D318" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.336805555555</v>
+      </c>
+      <c r="E318" t="s">
+        <v>329</v>
+      </c>
+      <c r="G318" t="s">
+        <v>487</v>
+      </c>
+      <c r="H318" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="319" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A319" t="s">
+        <v>8</v>
+      </c>
+      <c r="B319" s="1">
+        <v>46308.336805555547</v>
+      </c>
+      <c r="C319" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D319" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.347222222212</v>
+      </c>
+      <c r="E319" t="s">
+        <v>517</v>
+      </c>
+      <c r="G319" t="s">
+        <v>487</v>
+      </c>
+      <c r="H319" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="320" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A320" t="s">
+        <v>8</v>
+      </c>
+      <c r="B320" s="1">
+        <v>46308.347222222219</v>
+      </c>
+      <c r="C320" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D320" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.357638888883</v>
+      </c>
+      <c r="E320" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A321" t="s">
+        <v>12</v>
+      </c>
+      <c r="B321" s="1">
+        <v>46308.354166666664</v>
+      </c>
+      <c r="C321" s="3">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D321" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.375</v>
+      </c>
+      <c r="E321" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A322" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B322" s="7">
+        <v>46308.375</v>
+      </c>
+      <c r="C322" s="8">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D322" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.416666666664</v>
+      </c>
+      <c r="E322" s="9" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A323" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="B323" s="7">
+        <v>46308.416666666664</v>
+      </c>
+      <c r="C323" s="8">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D323" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.4375</v>
+      </c>
+      <c r="E323" s="6" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A324" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="B324" s="7">
+        <v>46308.527777777781</v>
+      </c>
+      <c r="C324" s="8">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D324" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.534722222226</v>
+      </c>
+      <c r="E324" s="6" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A325" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B325" s="7">
+        <v>46308.625</v>
+      </c>
+      <c r="C325" s="8">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D325" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.645833333336</v>
+      </c>
+      <c r="E325" s="9" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A326" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B326" s="7">
+        <v>46308.645833333336</v>
+      </c>
+      <c r="C326" s="8">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D326" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.666666666672</v>
+      </c>
+      <c r="E326" s="9" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A327" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B327" s="7">
+        <v>46308.645833333336</v>
+      </c>
+      <c r="C327" s="8">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D327" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.666666666672</v>
+      </c>
+      <c r="E327" s="9" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A328" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="B328" s="7">
+        <v>46308.666666666664</v>
+      </c>
+      <c r="C328" s="8">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D328" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46308.708333333328</v>
+      </c>
+      <c r="E328" s="9" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A329" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="B329" s="7">
+        <v>46309.3125</v>
+      </c>
+      <c r="C329" s="8">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D329" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46309.326388888891</v>
+      </c>
+      <c r="E329" s="6" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A330" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B330" s="7">
+        <v>46309.326388888891</v>
+      </c>
+      <c r="C330" s="8">
+        <v>3.125E-2</v>
+      </c>
+      <c r="D330" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46309.357638888891</v>
+      </c>
+      <c r="E330" s="9" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A331" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B331" s="7">
+        <v>46309.357638888891</v>
+      </c>
+      <c r="C331" s="8">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D331" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46309.378472222226</v>
+      </c>
+      <c r="E331" s="9" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A332" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B332" s="7">
+        <v>46309.378472222219</v>
+      </c>
+      <c r="C332" s="8">
+        <v>1.7361111111111112E-2</v>
+      </c>
+      <c r="D332" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46309.395833333328</v>
+      </c>
+      <c r="E332" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A333" t="s">
+        <v>8</v>
+      </c>
+      <c r="B333" s="1">
+        <v>46309.395833333336</v>
+      </c>
+      <c r="C333" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D333" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46309.402777777781</v>
+      </c>
+      <c r="E333" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A334" t="s">
+        <v>8</v>
+      </c>
+      <c r="B334" s="1">
+        <v>46309.402777777781</v>
+      </c>
+      <c r="C334" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D334" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46309.409722222226</v>
+      </c>
+      <c r="E334" t="s">
+        <v>533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
20_usuarios_dimensionado archivo semana 19-25 octubre y worklog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -224,8 +224,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H350" headerRowCount="1" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:H350"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H369" headerRowCount="1" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+  <autoFilter ref="A1:H369"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Ticket"/>
     <tableColumn id="2" name="Fecha" dataDxfId="2"/>
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H350"/>
+  <dimension ref="A1:H369"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="18.140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -12110,6 +12110,639 @@
       <c r="H350" t="inlineStr">
         <is>
           <t>523847</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>DSS-9780</t>
+        </is>
+      </c>
+      <c r="B351" s="1" t="n">
+        <v>46310.31597222222</v>
+      </c>
+      <c r="C351" s="3" t="n">
+        <v>0.05902777777777778</v>
+      </c>
+      <c r="D351" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E351" s="5" t="inlineStr">
+        <is>
+          <t>Creación de archivo multimétrico</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>524456</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="6" t="inlineStr">
+        <is>
+          <t>DSS-9337</t>
+        </is>
+      </c>
+      <c r="B352" s="7" t="n">
+        <v>46310.375</v>
+      </c>
+      <c r="C352" s="8" t="n">
+        <v>0.02083333333333333</v>
+      </c>
+      <c r="D352" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E352" s="6" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>524457</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>DSS-9780</t>
+        </is>
+      </c>
+      <c r="B353" s="1" t="n">
+        <v>46310.39583333334</v>
+      </c>
+      <c r="C353" s="3" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="D353" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E353" s="5" t="inlineStr">
+        <is>
+          <t>Creación de archivo multimétrico</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>524458</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>DSS-9780</t>
+        </is>
+      </c>
+      <c r="B354" s="1" t="n">
+        <v>46310.625</v>
+      </c>
+      <c r="C354" s="3" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="D354" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E354" s="5" t="inlineStr">
+        <is>
+          <t>Creación de archivo multimétrico</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr"/>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>524459</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>DSS-9337</t>
+        </is>
+      </c>
+      <c r="B355" s="1" t="n">
+        <v>46310.66666666666</v>
+      </c>
+      <c r="C355" s="3" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="D355" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Seguimiento Reestructuración Ecosistema Reporting</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr"/>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>524321</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B356" s="1" t="n">
+        <v>46311.27083333334</v>
+      </c>
+      <c r="C356" s="3" t="n">
+        <v>0.003472222222222222</v>
+      </c>
+      <c r="D356" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Descarga insumos SF</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr"/>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>524322</t>
+        </is>
+      </c>
+    </row>
+    <row r="357" ht="30" customHeight="1">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>DSS-9780</t>
+        </is>
+      </c>
+      <c r="B357" s="1" t="n">
+        <v>46311.27430555555</v>
+      </c>
+      <c r="C357" s="3" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="D357" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E357" s="5" t="inlineStr">
+        <is>
+          <t>Se actualizó el archivo con los indicadores del mes de setiembre y octubre.
+Se revisó que las referencias sean las correctas a la fuente</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr"/>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>524323</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B358" s="1" t="n">
+        <v>46311.31597222222</v>
+      </c>
+      <c r="C358" s="3" t="n">
+        <v>0.05902777777777778</v>
+      </c>
+      <c r="D358" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Actualización CDM</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr"/>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>524460</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="6" t="inlineStr">
+        <is>
+          <t>DSS-9337</t>
+        </is>
+      </c>
+      <c r="B359" s="7" t="n">
+        <v>46311.375</v>
+      </c>
+      <c r="C359" s="8" t="n">
+        <v>0.01388888888888889</v>
+      </c>
+      <c r="D359" s="8">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E359" s="6" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr"/>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>524324</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B360" s="1" t="n">
+        <v>46311.38888888889</v>
+      </c>
+      <c r="C360" s="3" t="n">
+        <v>0.04513888888888889</v>
+      </c>
+      <c r="D360" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Actualización CDM</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr"/>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>524461</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B361" s="1" t="n">
+        <v>46311.43402777778</v>
+      </c>
+      <c r="C361" s="3" t="n">
+        <v>0.006944444444444444</v>
+      </c>
+      <c r="D361" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>ISN</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr"/>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>524325</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B362" s="1" t="n">
+        <v>46281.44097222222</v>
+      </c>
+      <c r="C362" s="3" t="n">
+        <v>0.01388888888888889</v>
+      </c>
+      <c r="D362" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Envío dimensionado</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr"/>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>524462</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B363" s="1" t="n">
+        <v>46281.45486111111</v>
+      </c>
+      <c r="C363" s="3" t="n">
+        <v>0.01388888888888889</v>
+      </c>
+      <c r="D363" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Comisiones</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr"/>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>524463</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>DSS-9797</t>
+        </is>
+      </c>
+      <c r="B364" s="1" t="n">
+        <v>46281.46875</v>
+      </c>
+      <c r="C364" s="3" t="n">
+        <v>0.02083333333333333</v>
+      </c>
+      <c r="D364" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Revision de datos y lógica del proceso.</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr"/>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>524326</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B365" s="1" t="n">
+        <v>46281.48958333334</v>
+      </c>
+      <c r="C365" s="3" t="n">
+        <v>0.02777777777777778</v>
+      </c>
+      <c r="D365" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Impacto parque 202609</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr"/>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>524327</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>DSS-9841</t>
+        </is>
+      </c>
+      <c r="B366" s="1" t="n">
+        <v>46281.51736111111</v>
+      </c>
+      <c r="C366" s="3" t="n">
+        <v>0.06597222222222222</v>
+      </c>
+      <c r="D366" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Desarrollo de solicitud</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr"/>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>524464</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>DSS-9841</t>
+        </is>
+      </c>
+      <c r="B367" s="1" t="n">
+        <v>46281.625</v>
+      </c>
+      <c r="C367" s="3" t="n">
+        <v>0.09375</v>
+      </c>
+      <c r="D367" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Desarrollo de solicitud</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr"/>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Sí (16/10/2026 17:14)</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>524465</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B368" s="1" t="n">
+        <v>46314.27083333334</v>
+      </c>
+      <c r="C368" s="3" t="n">
+        <v>0.003472222222222222</v>
+      </c>
+      <c r="D368" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Descarga insumos SF</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr"/>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Sí (19/10/2026 08:26)</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>524562</t>
+        </is>
+      </c>
+    </row>
+    <row r="369" ht="90" customHeight="1">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>DSS-9848</t>
+        </is>
+      </c>
+      <c r="B369" s="1" t="n">
+        <v>46314.27430555555</v>
+      </c>
+      <c r="C369" s="3" t="n">
+        <v>0.05902777777777778</v>
+      </c>
+      <c r="D369" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E369" s="5" t="inlineStr">
+        <is>
+          <t>Se realizó lo siguiente:
+Revision de proceso ETL
+Revisión de archivos fisicos
+Redireccion a nueva columa
+Corrida el proceso
+Corrida de los diferentes informes.</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr"/>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Sí (19/10/2026 08:26)</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>524911</t>
         </is>
       </c>
     </row>

</xml_diff>